<commit_message>
update cbm result table konte
</commit_message>
<xml_diff>
--- a/analysis/CBM/2025/Konte/data/CBM_format/IN1020_2025_CBM_konte_results.xlsx
+++ b/analysis/CBM/2025/Konte/data/CBM_format/IN1020_2025_CBM_konte_results.xlsx
@@ -637,25 +637,53 @@
       <c r="E4" t="n">
         <v>8</v>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="G4" t="n">
         <v>8</v>
       </c>
       <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="M4" t="n">
         <v>8</v>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="O4" t="n">
         <v>8</v>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="Q4" t="n">
         <v>56</v>
       </c>
@@ -750,7 +778,11 @@
       <c r="L6" t="n">
         <v>8</v>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="N6" t="n">
         <v>4</v>
       </c>
@@ -933,7 +965,11 @@
       <c r="C10" t="n">
         <v>8</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="E10" t="n">
         <v>8</v>
       </c>
@@ -946,14 +982,22 @@
       <c r="H10" t="n">
         <v>4</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="J10" t="n">
         <v>-12</v>
       </c>
       <c r="K10" t="n">
         <v>-12</v>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="M10" t="n">
         <v>4</v>
       </c>
@@ -1192,7 +1236,11 @@
       <c r="C15" t="n">
         <v>-2</v>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="E15" t="n">
         <v>8</v>
       </c>
@@ -1208,7 +1256,11 @@
       <c r="I15" t="n">
         <v>8</v>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="K15" t="n">
         <v>2</v>
       </c>
@@ -1288,7 +1340,11 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="C17" t="n">
         <v>8</v>
       </c>
@@ -1946,7 +2002,11 @@
       <c r="I29" t="n">
         <v>6</v>
       </c>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="K29" t="n">
         <v>8</v>
       </c>
@@ -2430,7 +2490,11 @@
       <c r="L38" t="n">
         <v>6</v>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="N38" t="n">
         <v>7</v>
       </c>
@@ -3196,7 +3260,11 @@
       <c r="C53" t="n">
         <v>8</v>
       </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="E53" t="n">
         <v>8</v>
       </c>
@@ -3227,7 +3295,11 @@
       <c r="N53" t="n">
         <v>8</v>
       </c>
-      <c r="O53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="P53" t="n">
         <v>8</v>
       </c>
@@ -3504,25 +3576,77 @@
       <c r="A59" t="n">
         <v>58</v>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="E59" t="n">
         <v>4</v>
       </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="M59" t="n">
         <v>-12</v>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="Q59" t="n">
         <v>-8</v>
       </c>
@@ -3690,23 +3814,79 @@
       <c r="A63" t="n">
         <v>62</v>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="E63" t="n">
         <v>8</v>
       </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="Q63" t="n">
         <v>8</v>
       </c>
@@ -3810,7 +3990,11 @@
       <c r="O65" t="n">
         <v>8</v>
       </c>
-      <c r="P65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
       <c r="Q65" t="n">
         <v>72</v>
       </c>

</xml_diff>

<commit_message>
konte resulta without F
</commit_message>
<xml_diff>
--- a/analysis/CBM/2025/Konte/data/CBM_format/IN1020_2025_CBM_konte_results.xlsx
+++ b/analysis/CBM/2025/Konte/data/CBM_format/IN1020_2025_CBM_konte_results.xlsx
@@ -553,7 +553,7 @@
         <v>8</v>
       </c>
       <c r="M2" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N2" t="n">
         <v>4</v>
@@ -565,7 +565,7 @@
         <v>8</v>
       </c>
       <c r="Q2" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
@@ -612,13 +612,13 @@
         <v>8</v>
       </c>
       <c r="O3" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>8</v>
       </c>
       <c r="Q3" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -834,7 +834,7 @@
         <v>8</v>
       </c>
       <c r="M7" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N7" t="n">
         <v>8</v>
@@ -846,7 +846,7 @@
         <v>8</v>
       </c>
       <c r="Q7" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8">
@@ -940,7 +940,7 @@
         <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N9" t="n">
         <v>7</v>
@@ -952,7 +952,7 @@
         <v>8</v>
       </c>
       <c r="Q9" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10">
@@ -977,7 +977,7 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>4</v>
@@ -1011,7 +1011,7 @@
         <v>8</v>
       </c>
       <c r="Q10" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
@@ -1105,7 +1105,7 @@
         <v>8</v>
       </c>
       <c r="M12" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>4</v>
@@ -1117,7 +1117,7 @@
         <v>4</v>
       </c>
       <c r="Q12" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1262,10 +1262,10 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
         <v>5</v>
@@ -1280,7 +1280,7 @@
         <v>7</v>
       </c>
       <c r="Q15" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16">
@@ -1321,7 +1321,7 @@
         <v>8</v>
       </c>
       <c r="M16" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N16" t="n">
         <v>8</v>
@@ -1333,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="Q16" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17">
@@ -1385,10 +1385,10 @@
         <v>8</v>
       </c>
       <c r="P17" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18">
@@ -1396,7 +1396,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" t="n">
         <v>8</v>
@@ -1441,7 +1441,7 @@
         <v>6</v>
       </c>
       <c r="Q18" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19">
@@ -1588,7 +1588,7 @@
         <v>8</v>
       </c>
       <c r="M21" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>7</v>
@@ -1600,7 +1600,7 @@
         <v>8</v>
       </c>
       <c r="Q21" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22">
@@ -1614,13 +1614,13 @@
         <v>6</v>
       </c>
       <c r="D22" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
         <v>8</v>
       </c>
       <c r="F22" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>8</v>
@@ -1647,13 +1647,13 @@
         <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="P22" t="n">
         <v>6</v>
       </c>
       <c r="Q22" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23">
@@ -1694,7 +1694,7 @@
         <v>8</v>
       </c>
       <c r="M23" t="n">
-        <v>-9</v>
+        <v>2</v>
       </c>
       <c r="N23" t="n">
         <v>8</v>
@@ -1703,10 +1703,10 @@
         <v>6</v>
       </c>
       <c r="P23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q23" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24">
@@ -1717,13 +1717,13 @@
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" t="n">
         <v>-12</v>
       </c>
       <c r="E24" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
@@ -1747,7 +1747,7 @@
         <v>8</v>
       </c>
       <c r="M24" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>8</v>
@@ -1759,7 +1759,7 @@
         <v>8</v>
       </c>
       <c r="Q24" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25">
@@ -1853,7 +1853,7 @@
         <v>8</v>
       </c>
       <c r="M26" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>8</v>
@@ -1865,7 +1865,7 @@
         <v>4</v>
       </c>
       <c r="Q26" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27">
@@ -1932,13 +1932,13 @@
         <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>-9</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>8</v>
       </c>
       <c r="F28" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G28" t="n">
         <v>8</v>
@@ -1959,7 +1959,7 @@
         <v>4</v>
       </c>
       <c r="M28" t="n">
-        <v>-9</v>
+        <v>2</v>
       </c>
       <c r="N28" t="n">
         <v>6</v>
@@ -1968,10 +1968,10 @@
         <v>6</v>
       </c>
       <c r="P28" t="n">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>37</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29">
@@ -2120,7 +2120,7 @@
         <v>6</v>
       </c>
       <c r="M31" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N31" t="n">
         <v>6</v>
@@ -2132,7 +2132,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32">
@@ -2158,34 +2158,34 @@
         <v>8</v>
       </c>
       <c r="H32" t="n">
+        <v>4</v>
+      </c>
+      <c r="I32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>6</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L32" t="n">
+        <v>8</v>
+      </c>
+      <c r="M32" t="n">
+        <v>8</v>
+      </c>
+      <c r="N32" t="n">
+        <v>8</v>
+      </c>
+      <c r="O32" t="n">
+        <v>8</v>
+      </c>
+      <c r="P32" t="n">
         <v>3</v>
       </c>
-      <c r="I32" t="n">
-        <v>8</v>
-      </c>
-      <c r="J32" t="n">
-        <v>6</v>
-      </c>
-      <c r="K32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" t="n">
-        <v>8</v>
-      </c>
-      <c r="M32" t="n">
-        <v>8</v>
-      </c>
-      <c r="N32" t="n">
-        <v>8</v>
-      </c>
-      <c r="O32" t="n">
-        <v>8</v>
-      </c>
-      <c r="P32" t="n">
-        <v>2</v>
-      </c>
       <c r="Q32" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33">
@@ -2193,7 +2193,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
         <v>6</v>
@@ -2208,7 +2208,7 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
         <v>8</v>
@@ -2226,7 +2226,7 @@
         <v>4</v>
       </c>
       <c r="M33" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
         <v>6</v>
@@ -2235,10 +2235,10 @@
         <v>4</v>
       </c>
       <c r="P33" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="Q33" t="n">
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34">
@@ -2261,7 +2261,7 @@
         <v>6</v>
       </c>
       <c r="G34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H34" t="n">
         <v>5</v>
@@ -2276,7 +2276,7 @@
         <v>4</v>
       </c>
       <c r="L34" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="M34" t="n">
         <v>5</v>
@@ -2285,13 +2285,13 @@
         <v>7</v>
       </c>
       <c r="O34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P34" t="n">
         <v>5</v>
       </c>
       <c r="Q34" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35">
@@ -2332,7 +2332,7 @@
         <v>8</v>
       </c>
       <c r="M35" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>-12</v>
@@ -2341,10 +2341,10 @@
         <v>8</v>
       </c>
       <c r="P35" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>24</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36">
@@ -2364,7 +2364,7 @@
         <v>8</v>
       </c>
       <c r="F36" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
         <v>-2</v>
@@ -2382,13 +2382,13 @@
         <v>8</v>
       </c>
       <c r="L36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -2397,7 +2397,7 @@
         <v>4</v>
       </c>
       <c r="Q36" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37">
@@ -2435,10 +2435,10 @@
         <v>8</v>
       </c>
       <c r="L37" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N37" t="n">
         <v>6</v>
@@ -2447,10 +2447,10 @@
         <v>8</v>
       </c>
       <c r="P37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q37" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38">
@@ -2546,7 +2546,7 @@
         <v>8</v>
       </c>
       <c r="M39" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>8</v>
@@ -2555,10 +2555,10 @@
         <v>8</v>
       </c>
       <c r="P39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q39" t="n">
-        <v>71</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40">
@@ -2572,7 +2572,7 @@
         <v>8</v>
       </c>
       <c r="D40" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
         <v>8</v>
@@ -2581,7 +2581,7 @@
         <v>8</v>
       </c>
       <c r="G40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H40" t="n">
         <v>6</v>
@@ -2611,7 +2611,7 @@
         <v>0</v>
       </c>
       <c r="Q40" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41">
@@ -2672,7 +2672,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
         <v>4</v>
@@ -2702,10 +2702,10 @@
         <v>8</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
         <v>5</v>
@@ -2717,7 +2717,7 @@
         <v>6</v>
       </c>
       <c r="Q42" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43">
@@ -2793,7 +2793,7 @@
         <v>4</v>
       </c>
       <c r="G44" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
         <v>4</v>
@@ -2808,7 +2808,7 @@
         <v>8</v>
       </c>
       <c r="L44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M44" t="n">
         <v>7</v>
@@ -2823,7 +2823,7 @@
         <v>8</v>
       </c>
       <c r="Q44" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
     </row>
     <row r="45">
@@ -2864,7 +2864,7 @@
         <v>8</v>
       </c>
       <c r="M45" t="n">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
         <v>8</v>
@@ -2876,7 +2876,7 @@
         <v>8</v>
       </c>
       <c r="Q45" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46">
@@ -2905,7 +2905,7 @@
         <v>7</v>
       </c>
       <c r="I46" t="n">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="J46" t="n">
         <v>8</v>
@@ -2926,10 +2926,10 @@
         <v>6</v>
       </c>
       <c r="P46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q46" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47">
@@ -3032,10 +3032,10 @@
         <v>7</v>
       </c>
       <c r="P48" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="Q48" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49">
@@ -3161,7 +3161,7 @@
         <v>8</v>
       </c>
       <c r="F51" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="G51" t="n">
         <v>8</v>
@@ -3173,7 +3173,7 @@
         <v>3</v>
       </c>
       <c r="J51" t="n">
-        <v>-9</v>
+        <v>2</v>
       </c>
       <c r="K51" t="n">
         <v>8</v>
@@ -3182,10 +3182,10 @@
         <v>8</v>
       </c>
       <c r="M51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N51" t="n">
-        <v>-9</v>
+        <v>2</v>
       </c>
       <c r="O51" t="n">
         <v>4</v>
@@ -3194,7 +3194,7 @@
         <v>8</v>
       </c>
       <c r="Q51" t="n">
-        <v>51</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52">
@@ -3232,7 +3232,7 @@
         <v>8</v>
       </c>
       <c r="L52" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="M52" t="n">
         <v>6</v>
@@ -3247,7 +3247,7 @@
         <v>8</v>
       </c>
       <c r="Q52" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="53">
@@ -3290,7 +3290,7 @@
         <v>8</v>
       </c>
       <c r="M53" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N53" t="n">
         <v>8</v>
@@ -3304,7 +3304,7 @@
         <v>8</v>
       </c>
       <c r="Q53" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54">
@@ -3345,7 +3345,7 @@
         <v>8</v>
       </c>
       <c r="M54" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="N54" t="n">
         <v>8</v>
@@ -3357,7 +3357,7 @@
         <v>5</v>
       </c>
       <c r="Q54" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55">
@@ -3398,19 +3398,19 @@
         <v>8</v>
       </c>
       <c r="M55" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="N55" t="n">
         <v>6</v>
       </c>
       <c r="O55" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="P55" t="n">
         <v>6</v>
       </c>
       <c r="Q55" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56">
@@ -3451,7 +3451,7 @@
         <v>8</v>
       </c>
       <c r="M56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N56" t="n">
         <v>8</v>
@@ -3463,7 +3463,7 @@
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57">
@@ -3474,7 +3474,7 @@
         <v>4</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" t="n">
         <v>8</v>
@@ -3483,28 +3483,28 @@
         <v>8</v>
       </c>
       <c r="F57" t="n">
+        <v>3</v>
+      </c>
+      <c r="G57" t="n">
+        <v>4</v>
+      </c>
+      <c r="H57" t="n">
+        <v>6</v>
+      </c>
+      <c r="I57" t="n">
+        <v>5</v>
+      </c>
+      <c r="J57" t="n">
+        <v>4</v>
+      </c>
+      <c r="K57" t="n">
+        <v>8</v>
+      </c>
+      <c r="L57" t="n">
         <v>2</v>
       </c>
-      <c r="G57" t="n">
-        <v>-2</v>
-      </c>
-      <c r="H57" t="n">
-        <v>6</v>
-      </c>
-      <c r="I57" t="n">
-        <v>5</v>
-      </c>
-      <c r="J57" t="n">
-        <v>4</v>
-      </c>
-      <c r="K57" t="n">
-        <v>8</v>
-      </c>
-      <c r="L57" t="n">
-        <v>-4</v>
-      </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N57" t="n">
         <v>6</v>
@@ -3516,7 +3516,7 @@
         <v>4</v>
       </c>
       <c r="Q57" t="n">
-        <v>56</v>
+        <v>71</v>
       </c>
     </row>
     <row r="58">
@@ -3668,10 +3668,10 @@
         <v>8</v>
       </c>
       <c r="F60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H60" t="n">
         <v>6</v>
@@ -3689,19 +3689,19 @@
         <v>7</v>
       </c>
       <c r="M60" t="n">
+        <v>4</v>
+      </c>
+      <c r="N60" t="n">
+        <v>5</v>
+      </c>
+      <c r="O60" t="n">
+        <v>8</v>
+      </c>
+      <c r="P60" t="n">
         <v>3</v>
       </c>
-      <c r="N60" t="n">
-        <v>5</v>
-      </c>
-      <c r="O60" t="n">
-        <v>8</v>
-      </c>
-      <c r="P60" t="n">
-        <v>2</v>
-      </c>
       <c r="Q60" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61">
@@ -3721,7 +3721,7 @@
         <v>8</v>
       </c>
       <c r="F61" t="n">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
         <v>8</v>
@@ -3748,13 +3748,13 @@
         <v>4</v>
       </c>
       <c r="O61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P61" t="n">
         <v>7</v>
       </c>
       <c r="Q61" t="n">
-        <v>62</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62">
@@ -3911,7 +3911,7 @@
         <v>-6</v>
       </c>
       <c r="G64" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H64" t="n">
         <v>7</v>
@@ -3941,7 +3941,7 @@
         <v>7</v>
       </c>
       <c r="Q64" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65">
@@ -3964,7 +3964,7 @@
         <v>4</v>
       </c>
       <c r="G65" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
         <v>8</v>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>72</v>
+        <v>88</v>
       </c>
     </row>
     <row r="66">
@@ -4037,7 +4037,7 @@
         <v>7</v>
       </c>
       <c r="M66" t="n">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="N66" t="n">
         <v>8</v>
@@ -4049,7 +4049,7 @@
         <v>7</v>
       </c>
       <c r="Q66" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="67">
@@ -4063,7 +4063,7 @@
         <v>8</v>
       </c>
       <c r="D67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E67" t="n">
         <v>8</v>
@@ -4102,7 +4102,7 @@
         <v>8</v>
       </c>
       <c r="Q67" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="68">

</xml_diff>